<commit_message>
Faz 4: ilk etiketleme (kural netleştirme öncesi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gold/etiketleme.xlsx
+++ b/data/gold/etiketleme.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +11,7 @@
     <sheet name="Yedekler" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,12 +27,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -45,17 +49,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A5F"/>
+        <fgColor rgb="FF1F3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF4CC"/>
+        <fgColor rgb="FFFFF4CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,15 +84,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -452,20 +456,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ETİKETLEME TALİMATI</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,9 +482,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -526,9 +524,6 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -585,9 +580,6 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -602,9 +594,6 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -618,9 +607,6 @@
           <t xml:space="preserve">        -&gt; gap_var = Evet | Malzeme = X (su geçirmezlik malzeme iddiası) | seviye = Yüksek | not: 'Su geçirmez diyor, 2/2 ilgili yorum su aldı diyor'</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -641,26 +627,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="75" customWidth="1" min="4" max="4"/>
+    <col width="117.5" customWidth="1" min="3" max="3"/>
+    <col width="152" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="6" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="35" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -737,7 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="300" customHeight="1">
+    <row r="2" ht="272" customHeight="1">
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
@@ -772,19 +751,39 @@
 6) [1★] Way Too SMALL!! — Way too small, save your money, buy a different brand. I thought I got a great deal and purchased MULTIPLE white and black sets for my two boys, already opened all but one of them so it's too late to return them...save yourself. I wear size 10 men's and these are snug on me.</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="n"/>
-      <c r="N2" s="5" t="n"/>
-      <c r="O2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="300" customHeight="1">
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "15-18 numara için gerçek XXL" vaadine karşılık, 5 farklı yorum çorapların çok küçük olduğunu ve 10-13 numaralara bile dar geldiğini belirterek doğrudan iddiayı çürütmüştür. Fiyat şikayeti elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="409.6" customHeight="1">
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
@@ -828,19 +827,39 @@
 15) [1★] d. Used to be loyal to Rothco now it’s over priced junk — Rothco is wildly inconsistent. You could order 2 of the same product and receive different fits different materials. Don’t waste your money</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
-      <c r="N3" s="5" t="n"/>
-      <c r="O3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="300" customHeight="1">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "rahat" kargo pantolon vaadine ve sunduğu beden ölçülerine karşılık, 5 farklı yorum ürünün belirtilen bedenlerden çok küçük olduğunu ve "skinny jean" gibi aşırı dar bir kalıbı olduğunu belirterek iddiayı çürütmüştür. Fermuar, yıkamada çekme, kaşındıran kumaş ve eksik parça (sadece pantolon gelmesi) şikayetleri "en az 2" kuralını sağlamadığı için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
@@ -874,19 +893,43 @@
 8) [1★] Sequins catch — Sequins catch on each other when walking.</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="300" customHeight="1">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "esnek, bedeni saran slim kalıp" ve "parti taytı" vaatlerine karşılık; 6 yorum pulların birbirine takıldığını, döküldüğünü ve bedeni çizdiğini (Kalite), 3 yorum ise kalıbın sarmadığını, belin gevşek ve ağın orantısız uzun olduğunu (Beden/Kalıp) belirterek iddiaları çürütmüştür. Tekil dikiş söküğü şikayeti elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
@@ -917,19 +960,39 @@
 3) [2★] Sock too small — Little baby socks for little doll people. What is this world coming to!?!?</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="300" customHeight="1">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Sayfada turuncu renk belirtilmişken, 2 yorum rengin çok soluk ve donuk olduğunu belirterek beklenti çelişkisi oluşturmuştur (Renk); çorabın küçük olduğuna dair tekil şikayet elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="409" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
@@ -972,19 +1035,43 @@
 15) [2★] Not short people friendly — This is not plus size short people friendly I kept having to pull the tights up all night. They were not fitted at all around my private area. it was lose and made it kept dragging down and showing weirdly under the dress. Not worth it at all.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="300" customHeight="1">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın büyük bedenler için "kısıtlama yapmayan esneklik ve tüm gün rahatlık" vaadine karşılık; 4 yorum ağ boyunun kısa ve kalıbın çok dar olduğunu (Beden/Kalıp), 2 yorum ise ürünün giyildiği ilk saatlerde/günde yırtıldığını (Dayanıklılık) belirterek iddiaları çürütmüştür. Yanlış renk gönderimi ve tekil dikiş detayı şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="409" customHeight="1">
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
@@ -1020,17 +1107,41 @@
 5) [1★] BAIT AND SWITCH — Listing mentions “save $4 with coupon”, then there is none.</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Sayfanın "uzun süreli kullanıma uygun, ferah ve klasik Crocs rahatlığı" vaatlerine karşılık; 2 yorum ürünün iç astarı olmaması ve sert yapısı nedeniyle bilek kemiklerine sürttüğünü, kanayan yaralara ve su toplamalarına yol açtığını (Beden/Kalıp, Kalite) belirterek iddiaları çürütmüştür. 1 aydan kısa sürede yıpranma, kupon eksikliği ve genel kalite düşüşü şikayetleri tekil kaldığı için elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="300" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -1058,19 +1169,47 @@
 5) [1★] Rip — Just received today, put them on and they are ripped on one side. 😕</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="300" customHeight="1">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın başlığındaki "Fleece" (polar) vaadine karşılık; 2 yorum ürünün polar olmadığını ve çok ince bir pamuklu olduğunu (Malzeme), 3 yorum ise ürünün giyildiği anda/ilk günde dikişlerinden yırtıldığını ve deliklerle geldiğini (Dayanıklılık/Kalite) belirterek iddiaları çürütmüştür. Tekil dar kalıp şikayeti elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="409" customHeight="1">
       <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
@@ -1104,19 +1243,35 @@
 3) [2★] Chuge!!!! — Definitely buy a size down. If not you can use it as a parachute. These are chuge!!!</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="300" customHeight="1">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="n"/>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Yorumlarda yakanın duruşu (Görsel), yıkamada çekme ve sökülme (Kalite/Dayanıklılık) ile kalıbın çok büyük olması (Beden/Kalıp) konularında tekil şikayetler mevcut, ancak hiçbiri "en az 2" kuralını sağlayacak kadar tekrarlanmadığı için sistematik bir çelişki tespit edilmemiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="304" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
@@ -1149,19 +1304,39 @@
 8) [2★] Button fell off — Button fell off when I tried to put it on.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="300" customHeight="1">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>3 farklı yorum, ürünün yaka kapama düğmesinin paketten çıkar çıkmaz veya ilk denemede hemen koptuğunu belirterek net bir işçilik/kalite sorununa işaret etmiştir (Kalite). Lekeli/kullanılmış ürün şikayetleri satıcı hatası olduğu için, diğer tekil rahatsızlık ve görünüm eleştirileri ise "en az 2" kuralını karşılamadığı için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="409.6" customHeight="1">
       <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
@@ -1196,19 +1371,43 @@
 4) [1★] Nope. — Terrible. Do yourself a favor and just don't.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="5" t="n"/>
-    </row>
-    <row r="12" ht="300" customHeight="1">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "yüksek kalite" vaadine ve sunduğu görsellere karşılık, 2 farklı müşteri gelen ürünün fotoğraftakine benzemediğini ve kalitesiz/tuhaf bir kumaşı olduğunu belirterek iddiaları çürütmüştür (Görsel, Kalite). Dar kalıp, kimyasal koku ve renk şikayetleri "en az 2" kuralını sağlamadığı için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="409.6" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
@@ -1252,17 +1451,53 @@
 15) [1★] not the size expected — the shirt is not a tall shirt. the 3x in size is ok but it is not tall</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "Relaxed fit, dayanıklı ve kanvas" vaatlerine karşılık; 7 yorum ürünün çok küçük/kısa olduğunu (Beden/Kalıp), 4 yorum anında yırtıldığını/dikişlerin kalitesizliğini (Dayanıklılık/Kalite), 2 yorum kağıt gibi olup kanvas olmadığını (Malzeme) ve 2 yorum rengin farklı/koyu geldiğini (Renk) belirterek temel iddiaları çürütmüştür</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="300" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1292,19 +1527,39 @@
 3) [1★] Runs very small but too wide straps — Size 9/10 women’s was actually 8. Gave them away.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5" t="n"/>
-      <c r="O13" s="5" t="n"/>
-    </row>
-    <row r="14" ht="300" customHeight="1">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>Sayfada kalıba dair bir bilgi verilmemiş olmasına rağmen, 3 farklı yorum terliğin tabanının küçük ancak üst bantlarının aşırı bol/geniş olduğunu belirterek ciddi bir kalıp orantısızlığı (Beden/Kalıp) raporlamıştır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="272" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
@@ -1334,19 +1589,39 @@
 4) [1★] Two different widths! — I was given two different widths of the shoe. Left was wide and right was standard.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="5" t="n"/>
-    </row>
-    <row r="15" ht="300" customHeight="1">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="4" t="n"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın rahatlık ve beden/genişlik uyumu vaatlerine karşılık, 3 farklı yorum ayakkabının beklenen numaralardan çok daha küçük olduğunu belirterek iddiayı çürütmüştür (Beden/Kalıp). Yastıklama eksikliği şikayeti tekil kaldığı, yanlış eşleştirilmiş genişlik şikayeti ise satıcı hatası olduğu için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="272" customHeight="1">
       <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
@@ -1379,17 +1654,41 @@
 7) [2★] :( — It hasn't being a year and the leather cracked.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5" t="n"/>
-      <c r="O15" s="5" t="n"/>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "%100 Deri" ve hareketli yaşama uygunluk vaatlerine karşılık; 4 farklı yorum derinin çok kısa sürede (1.5 - 2 ay) çatladığını ve yırtıldığını (Dayanıklılık), 3 yorum ise ayakkabının çok sert, ağır ve rahatsız olduğunu (Kalite) belirterek temel iddiaları çürütmüştür. Tekil kalıp (büyük) şikayeti elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="300" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1422,19 +1721,39 @@
 4) [2★] Beautiful Shoes — These shoes just weren't right for me. I have a narrow foot and the straps across the front of the foot were too loose. These shoes also run small. I normally wear a 6 to 6.5 and needed a 7 in them. If I had ordered a 7 then the straps across the front would have been even more loose. I so wish they would have fit because they are gorgeous shoes!!!</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
-      <c r="N16" s="5" t="n"/>
-      <c r="O16" s="5" t="n"/>
-    </row>
-    <row r="17" ht="300" customHeight="1">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
+      <c r="M16" s="4" t="n"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "tam kararında uyum (right amount of fit)" vaadine karşılık, 2 farklı müşteri ürünün kalıbının çok dar ve numarasının küçük olduğunu belirterek beklentiyi çürütmüştür (Beden/Kalıp). Ön kayışın bolluğu ve iade ücreti kesintisi şikayetleri tekil ve ürün dışı olduğu için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="288" customHeight="1">
       <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
@@ -1471,19 +1790,47 @@
 8) [1★] My Poor Girl — Her booty hung out of every pair of these they were the worst</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5" t="n"/>
-      <c r="O17" s="5" t="n"/>
-    </row>
-    <row r="18" ht="300" customHeight="1">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="n"/>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın güvenlik amaçlı "vücudu saran kalıp (snug fit)" vaadine karşılık, 4 yorum ürünün kollarının/bacaklarının orantısız derecede kısa ve giyilemeyecek kadar küçük olduğunu (Beden/Kalıp); 2 yorum ise dikişlerin ilk birkaç kullanımda anında söküldüğünü (Dayanıklılık/Kalite) belirterek beklentileri tamamen çürütmüştür. Leke ve yıkama sonrası sarkma şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="409.6" customHeight="1">
       <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
@@ -1531,17 +1878,49 @@
 15) [1★] Ripped — Pants ripped after a few wears</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
-      <c r="L18" s="5" t="n"/>
-      <c r="M18" s="5" t="n"/>
-      <c r="N18" s="5" t="n"/>
-      <c r="O18" s="5" t="n"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="n"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "iç göstermez, derin squata uygun, dayanıklı ve destekleyici" vaatlerine karşılık; 8 yorum ürünün ilk kullanımlarda dikişlerinden yırtıldığını (Dayanıklılık), 3 yorum eğilirken tamamen iç gösterdiğini (Malzeme), 4 yorum kalıbın çok küçük olduğunu (Beden/Kalıp) ve 2 yorum sütyenin desteklemediğini (Kalite) belirterek tüm ana iddiaları çürütmüştür. Açık paket ve koku şikayetleri elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="300" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -1575,17 +1954,41 @@
 5) [1★] Straps — The straps doesn’t stick anymore. It was waste of money.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
-      <c r="M19" s="5" t="n"/>
-      <c r="N19" s="5" t="n"/>
-      <c r="O19" s="5" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "dayanıklı (durable)" yapı ve "gün boyu güvenli tutuş (secure fit)" sağlayan cırt cırt vaatlerine karşılık; 2 yorum ürünün ilk kullanımlarda koptuğunu/parçalandığını (Dayanıklılık), diğer 2 yorum ise cırt cırtların çok kısa sürede yapışkanlığını yitirdiğini (Kalite) belirterek temel iddiaları çürütmüştür. Tekil dar/uzun kalıp şikayeti elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="300" customHeight="1">
       <c r="A20" s="3" t="n">
@@ -1618,17 +2021,41 @@
 3) [1★] Horrible- save your money — They arrived in an airtight vacuum sealed bag and were perfect for my 5’ 6” grandson.</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
-      <c r="K20" s="5" t="n"/>
-      <c r="L20" s="5" t="n"/>
-      <c r="M20" s="5" t="n"/>
-      <c r="N20" s="5" t="n"/>
-      <c r="O20" s="5" t="n"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "aktif koşu pantolonu" ve "3 cep" vaatlerine karşılık; 3 yorum kalıbın aşırı küçük/orantısız olduğunu ve belden düştüğü için koşmayı engellediğini (Beden/Kalıp), 2 yorum ise ceplerin kullanılamayacak kadar küçük veya sahte olduğunu (Kalite) belirterek ana iddiaları çürütmüştür. Tekil malzeme (kağıt gibi dış kumaş) şikayeti elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="300" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1659,19 +2086,43 @@
 3) [2★] lasts a day in use wears out bottom — lasts a day in use wears out bottom</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
-      <c r="M21" s="5" t="n"/>
-      <c r="N21" s="5" t="n"/>
-      <c r="O21" s="5" t="n"/>
-    </row>
-    <row r="22" ht="300" customHeight="1">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın kauçuk tabanlı su ayakkabısı vaadine karşılık, 3 farklı yorum tabanın sadece 1-2 gün içinde delindiğini, aşındığını veya daha kullanılmadan iplerinin sökülerek parçalandığını (Dayanıklılık/Kalite) belirterek ürünün asgari işlevini çürütmüştür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="409.6" customHeight="1">
       <c r="A22" s="3" t="n">
         <v>21</v>
       </c>
@@ -1713,19 +2164,55 @@
 15) [2★] Sad — I got this hoodie about a month ago to surprise my boyfriend and the hoodie came in the mail with a hole in it. Had to throw it out and waste all that money:(</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="5" t="n"/>
-      <c r="K22" s="5" t="n"/>
-      <c r="L22" s="5" t="n"/>
-      <c r="M22" s="5" t="n"/>
-      <c r="N22" s="5" t="n"/>
-      <c r="O22" s="5" t="n"/>
-    </row>
-    <row r="23" ht="300" customHeight="1">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="n"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki "Loose Fit" ibaresine rağmen 3 yorum ürünün 1-2 beden daha büyük/orantısız olduğunu (Beden/Kalıp); 3 yorum rengin görseldekiyle ilgisi olmayıp neredeyse siyah renkte geldiğini (Renk/Görsel); 4 yorum ise dikişlerin çok özensiz olduğunu ve hemen sökülüp delindiğini (Kalite/Dayanıklılık) belirterek beklentileri çürütmüştür. Satıcı/yanlış ürün, koku ve haksız malzeme şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="335" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>22</v>
       </c>
@@ -1760,19 +2247,47 @@
 5) [2★] Already coming apart — I bought these about a week ago and wore them for the first time today. I just wore them around the house and for having them on for about half an hour, I noticed there was already a hole. The material is very cheap and i’m kind of disappointed. However, I guess you get what you pay for. I still expected more though. On the bright side, they are not itchy like a lot of shin/knee high socks are.</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="5" t="n"/>
-      <c r="M23" s="5" t="n"/>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="300" customHeight="1">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="n"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "dayanıklı yapı (durable construction)" vaadine karşılık; 2 yorum ürünün paketinden delik çıktığını veya yarım saatlik kullanımda delindiğini (Dayanıklılık/Kalite), 2 yorum da malzemenin çok ucuz ve ince olduğunu (Malzeme) belirterek ana iddiaları çürütmüştür. Tekil renk/desen ve dar baldır şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="380" customHeight="1">
       <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
@@ -1814,19 +2329,47 @@
 10) [1★] Poorly made and looks really cheap — This shirt is of extremely poor quality and not worth 50 plus dollars</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="5" t="n"/>
-      <c r="K24" s="5" t="n"/>
-      <c r="L24" s="5" t="n"/>
-      <c r="M24" s="5" t="n"/>
-      <c r="N24" s="5" t="n"/>
-      <c r="O24" s="5" t="n"/>
-    </row>
-    <row r="25" ht="300" customHeight="1">
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "premium pamuk" ve göğüs/omuzda "hafifçe dar (slightly slimmer) Custom Fit" vaatlerine karşılık; 4 yorum kalıbın aşırı küçük/orantısız olduğunu ve 3XL bedenin ancak bir çocuğa uyduğunu (Beden/Kalıp), 3 yorum ise kumaşın çok ucuz, ince ve kalitesiz hissettirdiğini (Kalite/Malzeme) belirterek ana iddiaları çürütmüştür. Satıcı hataları ve tekil renk şikayeti elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="409.6" customHeight="1">
       <c r="A25" s="3" t="n">
         <v>24</v>
       </c>
@@ -1868,17 +2411,45 @@
 15) [2★] Support — Not good support. Stretched out.</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
-      <c r="L25" s="5" t="n"/>
-      <c r="M25" s="5" t="n"/>
-      <c r="N25" s="5" t="n"/>
-      <c r="O25" s="5" t="n"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "dolgulu lüks iç taban" ve "olağanüstü konfor" vaatlerine karşılık; 3 yorum tabanın krep gibi dümdüz olduğunu ve hiçbir destek sunmadığını (Kalite), 5 yorum kalıbın aşırı küçük/orantısız olduğunu (Beden/Kalıp), 2 yorum kısa sürede esneyip şeklinin bozulduğunu (Dayanıklılık) belirterek ana iddiaları çürütmüştür. Eşitsiz ayakkabı (defolu ürün) ve iade sorunları elenmiştir</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="300" customHeight="1">
       <c r="A26" s="3" t="n">
@@ -1907,19 +2478,43 @@
 4) [2★] twisting elastic waist uncomfortable — the waist is much smaller than I anticipated (bought a large), and it fit more like a small. The elastic in the waist also keeps twisting and folding and is very uncomfortable.</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="n"/>
-      <c r="M26" s="5" t="n"/>
-      <c r="N26" s="5" t="n"/>
-      <c r="O26" s="5" t="n"/>
-    </row>
-    <row r="27" ht="300" customHeight="1">
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki temel spor eşofman takımı işlevine karşılık; 3 yorum bel lastiğinin sürekli kıvrıldığını, katlandığını veya ilk giyişte tamamen koptuğunu belirterek (Kalite/Dayanıklılık) ürünün asgari kullanım konforunu çürütmüştür. Tekil tüylenme/yıpranma ve dar beden şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="288" customHeight="1">
       <c r="A27" s="3" t="n">
         <v>26</v>
       </c>
@@ -1951,19 +2546,35 @@
 3) [1★] Missing Pieces to Set — My son has Prom coming up So i ordered ahead if time And half my items were missing from the order</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="5" t="n"/>
-      <c r="M27" s="5" t="n"/>
-      <c r="N27" s="5" t="n"/>
-      <c r="O27" s="5" t="n"/>
-    </row>
-    <row r="28" ht="300" customHeight="1">
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Yorumlarda paketlemeden kaynaklı eksik parça, sigara kokusu (kullanılmış ürün/satıcı hatası) ve aşırı küçük bel kalıbı gibi sorunlar dile getirilmiş olsa da, hiçbiri "en az 2" kuralını sağlayacak kadar tekrarlanmadığı için sistematik bir çelişki tespit edilmemiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="409.6" customHeight="1">
       <c r="A28" s="3" t="n">
         <v>27</v>
       </c>
@@ -2009,19 +2620,55 @@
 15) [1★] Not the same beautiful blue or good material quality as advertised &amp; viewed!! — Disliked color, quality of material &amp; cut! Cheap!!</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
-      <c r="L28" s="5" t="n"/>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="5" t="n"/>
-      <c r="O28" s="5" t="n"/>
-    </row>
-    <row r="29" ht="300" customHeight="1">
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "zarif, midi-boy yün kaban" vaadine karşılık; 4 yorum ürünün bir çocuk kabanı kadar küçük ve orantısız olduğunu (Beden/Kalıp), 4 yorum yanlış renk geldiğini (Renk), 6 yorum kumaşın çok ucuz, ince, sert ve kalitesiz olduğunu (Malzeme/Kalite), 2 yorum ise kesiminin ve duruşunun fotoğrafla hiç alakası olmadığını (Görsel) belirterek tüm temel iddiaları çürütmüştür. Kargo ve iade şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="320" customHeight="1">
       <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
@@ -2055,19 +2702,39 @@
 3) [2★] Too narrow, not fitting like other Clark's — Not a happy camper with these...to tight from the go, not at all fitting like my other Clark's. Immediately sent back</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="5" t="n"/>
-      <c r="K29" s="5" t="n"/>
-      <c r="L29" s="5" t="n"/>
-      <c r="M29" s="5" t="n"/>
-      <c r="N29" s="5" t="n"/>
-      <c r="O29" s="5" t="n"/>
-    </row>
-    <row r="30" ht="300" customHeight="1">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın konfor ve uyum (ayarlanabilir üst kısım) vaatlerine karşılık, 2 müşteri ayakkabının markanın diğer modellerine göre çok dar olduğunu ve ayağa iyi oturmadığını belirterek (Beden/Kalıp) beklentiyi çürütmüştür. İç tabanın çıkarılamaması şikayeti tekil olduğu için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="320" customHeight="1">
       <c r="A30" s="3" t="n">
         <v>29</v>
       </c>
@@ -2098,19 +2765,39 @@
 3) [1★] Careful--poor customer service/no resolution — I did not have a good experience with this company. The photo I submitted was "dark" (in retrospect) according to them but they went ahead and printed the pajamas. They should have asked for a different photo from me. As a result of their poor choice, my dog's brown hair is now an olive green over the entire set of pajamas! A green haired dog!!! Very disappointing. Also, the sizing runs small. Most mediums fit me fine but these sleeves were too short for my arms. They responded to this issue say</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
-      <c r="L30" s="5" t="n"/>
-      <c r="M30" s="5" t="n"/>
-      <c r="N30" s="5" t="n"/>
-      <c r="O30" s="5" t="n"/>
-    </row>
-    <row r="31" ht="300" customHeight="1">
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+      <c r="M30" s="4" t="n"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki "rahat kullanım" ve uygun kalıp vaadine karşılık; 2 farklı müşteri ürünün kalıbının çok küçük (2 beden dar) ve kollarının kısa olduğunu belirterek (Beden/Kalıp) beklentiyi çürütmüştür. Tekil malzeme (ucuz kumaş) ve yanlış baskı rengi (yeşil köpek) şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="395" customHeight="1">
       <c r="A31" s="3" t="n">
         <v>30</v>
       </c>
@@ -2150,19 +2837,43 @@
 11) [2★] Durability ssssssucks — They fell apart after 4 months of use</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
-      <c r="L31" s="5" t="n"/>
-      <c r="M31" s="5" t="n"/>
-      <c r="N31" s="5" t="n"/>
-      <c r="O31" s="5" t="n"/>
-    </row>
-    <row r="32" ht="300" customHeight="1">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "hafızalı sünger konforu" ve "yüksek kalite" vaatlerine karşılık; 2 yorum süngerin anında çökerek terliğin ayaktan çıkmasına/kramp yapmasına sebep olduğunu (Kalite), 3 yorum ise iç tabanların birkaç ay içinde yırtılıp ürünün parçalandığını (Dayanıklılık) belirterek ana iddiaları çürütmüştür. Satıcı, kullanılmış ürün ve tekil defo şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="408" customHeight="1">
       <c r="A32" s="3" t="n">
         <v>31</v>
       </c>
@@ -2201,17 +2912,45 @@
 8) [1★] Poor quality — I got the suite for my 23 m.o son, I got a size 3T, I thought it's kind of expensive and he can use it for 2 years or so. But he did wear it once for outside pool for 20 minutes and guess what...we got 2 big holes on the butt part of suite, it just felt apart...[...]oor quality, [...]wouldn/t recommend it to buy.</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="n"/>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="5" t="n"/>
-      <c r="K32" s="5" t="n"/>
-      <c r="L32" s="5" t="n"/>
-      <c r="M32" s="5" t="n"/>
-      <c r="N32" s="5" t="n"/>
-      <c r="O32" s="5" t="n"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="4" t="n"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "ilave sıcaklık sağlayan termal takım" vaadine karşılık; 4 yorum malzemenin çok ince olduğunu ve çocukların suda titreyip morardığını (Malzeme/Kalite), 4 yorum ise ürünün gövdeden çok kısa ve belden bol olacak şekilde orantısız bir kesime sahip olduğunu (Beden/Kalıp) belirterek temel iddiaları çürütmüştür. Tekil yırtılma şikayeti elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="300" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -2245,17 +2984,49 @@
 3) [1★] Pockets??? — This shirt has pockets on the front which are not visible in the ad. They are made of soft flimsy material which gives a messy look rather than clean lines. Otherwise, thee material is soft. Fits to size.</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
-      <c r="K33" s="5" t="n"/>
-      <c r="L33" s="5" t="n"/>
-      <c r="M33" s="5" t="n"/>
-      <c r="N33" s="5" t="n"/>
-      <c r="O33" s="5" t="n"/>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki görsel estetik beklentisine karşılık; 2 yorum rengin görseldeki gibi canlı olmadığını (Renk/Görsel), 3 yorum ise malzemenin çok ince, dayanıksız (flimsy) ve ucuz görünümlü olduğunu (Kalite/Malzeme) belirterek iddiaları çürütmüştür. Tekil gizli cep şikayeti elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="300" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -2285,19 +3056,35 @@
 3) [2★] Two Stars — Old shorts medium fit new shorts medium don't fit</t>
         </is>
       </c>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="5" t="n"/>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="5" t="n"/>
-      <c r="K34" s="5" t="n"/>
-      <c r="L34" s="5" t="n"/>
-      <c r="M34" s="5" t="n"/>
-      <c r="N34" s="5" t="n"/>
-      <c r="O34" s="5" t="n"/>
-    </row>
-    <row r="35" ht="300" customHeight="1">
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="n"/>
+      <c r="K34" s="4" t="n"/>
+      <c r="L34" s="4" t="n"/>
+      <c r="M34" s="4" t="n"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>Yorumlarda bir haftada taban ayrılması/parçalanma (Dayanıklılık), dar kalıp (Beden/Kalıp) ve yanlış ürüne yapılmış alakasız bir şort bedeni şikayeti bulunmasına rağmen, hiçbir şikayet "en az 2" kuralını sağlamadığı için sistematik bir çelişki tespit edilmemiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="409.6" customHeight="1">
       <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
@@ -2340,19 +3127,55 @@
 15) [1★] Not true to size — Hubby wears a 2x I ordered a 2x took it out n it immediately looked made small he tried it on n the length of a 2x came above his belt the shirt was definitely a 2x in width but a small in length</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="n"/>
-      <c r="K35" s="5" t="n"/>
-      <c r="L35" s="5" t="n"/>
-      <c r="M35" s="5" t="n"/>
-      <c r="N35" s="5" t="n"/>
-      <c r="O35" s="5" t="n"/>
-    </row>
-    <row r="36" ht="300" customHeight="1">
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "nefes alabilir, yumuşak kumaş" vaadine karşılık; 7 yorum kumaşın plastik gibi hissettirdiğini, nefes almadığını ve çok kalitesiz/ince olduğunu (Malzeme/Kalite), 4 yorum kalıpların standart dışı ve aşırı tutarsız (L'nin 3X, XXL'nin M gibi) olduğunu (Beden/Kalıp), 2 yorum ise rengin soluk/tozlu görünüp görselle uyuşmadığını (Renk/Görsel) belirterek ana iddiaları çürütmüştür. Kullanılmış ürün/satıcı şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="409.6" customHeight="1">
       <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
@@ -2394,19 +3217,39 @@
 15) [2★] too small! — Had to size up 2 sizes!!!</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
-      <c r="L36" s="5" t="n"/>
-      <c r="M36" s="5" t="n"/>
-      <c r="N36" s="5" t="n"/>
-      <c r="O36" s="5" t="n"/>
-    </row>
-    <row r="37" ht="300" customHeight="1">
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki "2 beden küçük kalıptır" uyarısına rağmen; incelenen 10 yorumun 10'u da kalıbın aşırı derecede küçük ve tutarsız olduğunu, 2 veya daha fazla beden büyük almanın bile ayakkabıyı giymek için yetersiz kaldığını (Beden/Kalıp) belirterek sayfanın temel beden yönlendirmesini çürütmüştür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="408" customHeight="1">
       <c r="A37" s="3" t="n">
         <v>36</v>
       </c>
@@ -2445,19 +3288,51 @@
 15) [1★] Go cotton! — Made my feet sweat and stink!</t>
         </is>
       </c>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="5" t="n"/>
-      <c r="L37" s="5" t="n"/>
-      <c r="M37" s="5" t="n"/>
-      <c r="N37" s="5" t="n"/>
-      <c r="O37" s="5" t="n"/>
-    </row>
-    <row r="38" ht="300" customHeight="1">
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "nefes alabilen file", "dayanıklı kumaş" ve "rahat uyum" vaatlerine karşılık; 8 yorum ürünün nem emmediğini, plastik poşet gibi terletip koku yaptığını (Malzeme/Kalite), 3 yorum bacakları aşırı sıktığını ve kalıpların tutarsız olduğunu (Beden/Kalıp), 3 yorum ise birkaç kullanımda delinip parçalandığını (Dayanıklılık) belirterek temel spor iddialarını çürütmüştür. Kargo ve okuma hatası şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="409.6" customHeight="1">
       <c r="A38" s="3" t="n">
         <v>37</v>
       </c>
@@ -2498,19 +3373,51 @@
 15) [2★] Buy at least one size bigger. — I normally wear a size 8 but I could barely get my foot into the sandal, I like the looks and feel of this sandal so I'm returning for a larger size.</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="5" t="n"/>
-      <c r="L38" s="5" t="n"/>
-      <c r="M38" s="5" t="n"/>
-      <c r="N38" s="5" t="n"/>
-      <c r="O38" s="5" t="n"/>
-    </row>
-    <row r="39" ht="300" customHeight="1">
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın konforlu adım ve dayanıklı kayış/taban vaatlerine karşılık; 8 yorum ürünün aşırı dar ve küçük olduğunu (Beden/Kalıp), 3 yorum kayış malzemesinin aşındırıcı olup ayağı soyduğunu (Malzeme/Kalite), 3 yorum ise tabanların haftalar/aylar içinde tamamen koptuğunu (Dayanıklılık) belirterek temel ürün işlevlerini çürütmüştür. İade ve koku şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="335" customHeight="1">
       <c r="A39" s="3" t="n">
         <v>38</v>
       </c>
@@ -2543,19 +3450,43 @@
 3) [1★] Literally the worst dress ever! — After trying this on for my husband he said, “please call Jedediah in from the barn.” It’s awful! The length is weird. The neck is too high. The sleeves are too puffy. The print is dated. I wanted to like this dress, but it lacks any redeeming qualities.</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
-      <c r="L39" s="5" t="n"/>
-      <c r="M39" s="5" t="n"/>
-      <c r="N39" s="5" t="n"/>
-      <c r="O39" s="5" t="n"/>
-    </row>
-    <row r="40" ht="300" customHeight="1">
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="n"/>
+      <c r="K39" s="4" t="n"/>
+      <c r="L39" s="4" t="n"/>
+      <c r="M39" s="4" t="n"/>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "vücut hatlarınızı gösteren A-kesim" ve "zarif duruş" vaatlerine karşılık; 2 yorum elbisenin tamamen şekilsiz, kutu gibi ve aşırı bol olduğunu (Beden/Kalıp), 2 yorum ise boyunun modeldekinden uzun ve tuhaf durduğunu (Görsel) belirterek temel estetik iddiaları çürütmüştür. Tekil yaka ve kol tasarımı şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="288" customHeight="1">
       <c r="A40" s="3" t="n">
         <v>39</v>
       </c>
@@ -2587,19 +3518,39 @@
 3) [1★] Size chart very misleading — Size chart is very misleading</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
-      <c r="L40" s="5" t="n"/>
-      <c r="M40" s="5" t="n"/>
-      <c r="N40" s="5" t="n"/>
-      <c r="O40" s="5" t="n"/>
-    </row>
-    <row r="41" ht="300" customHeight="1">
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="n"/>
+      <c r="K40" s="4" t="n"/>
+      <c r="L40" s="4" t="n"/>
+      <c r="M40" s="4" t="n"/>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "optimal destek sağlayan bel bandı" vaadine ve sunduğu beden ölçülerine karşılık; 3 yorum beden tablosunun tamamen yanıltıcı olduğunu, şortun aşırı küçük üretildiğini ve esnemeyen bel bandı yüzünden ürünün (örneğin 36 inç bele XL bedenin) kalçadan dahi geçmediğini (Beden/Kalıp) belirterek temel iddiaları çürütmüştür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="409" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>40</v>
       </c>
@@ -2631,24 +3582,41 @@
 3) [1★] Ugly as hell — It’s ugly , the fabric feet like a silk sheet .</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
-      <c r="L41" s="5" t="n"/>
-      <c r="M41" s="5" t="n"/>
-      <c r="N41" s="5" t="n"/>
-      <c r="O41" s="5" t="n"/>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="n"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="n"/>
+      <c r="M41" s="4" t="n"/>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki "%20 pamuklu, yumuşak tişört (tee)" vaadine karşılık; 2 farklı müşteri kumaşın standart bir tişört gibi olmadığını, parlak ve ipek çarşaf gibi (sentetik/silky) hissettirdiğini belirterek (Malzeme) beklentiyi çürütmüştür. Tekil dar beden ve fazla açık tasarım şikayetleri elenmiştir.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="E2:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Evet,Hayır"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="E2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Evet,Hayır"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:M41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2669,26 +3637,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="75" customWidth="1" min="4" max="4"/>
+    <col width="90.33203125" customWidth="1" min="3" max="3"/>
+    <col width="210" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="6" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="35" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -2765,7 +3726,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="300" customHeight="1">
+    <row r="2" ht="395" customHeight="1">
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
@@ -2799,19 +3760,47 @@
 13) [1★] One Star — Horrible horrible extremely small horrible material like flannel pajamas there was nothing attractive about this dress except the picture</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="n"/>
-      <c r="N2" s="5" t="n"/>
-      <c r="O2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="300" customHeight="1">
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "Diz Boyu Yetişkin Elbisesi (XL)" vaadine karşılık; 6 yorum elbisenin çok kısa olduğunu ve XL bedenin bir çocuğa veya M bedene uyacak kadar dar/küçük kalıplı olduğunu (Beden/Kalıp), 5 yorum ise malzemenin aşırı ince, uyduruk (flimsy) ve ucuz bir kostüm gibi hissettirdiğini (Malzeme/Kalite) belirterek ana iddiaları çürütmüştür. Genel memnuniyetsizlik belirten detaysız 1. yorum elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="272" customHeight="1">
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
@@ -2846,17 +3835,37 @@
 8) [1★] Awful quality — I had these shoes for one month and 11 days. I didn't wear them every day either. The heel on one shoe wore down to the metal stud almost immediately and the ankle strap snapped off of one. I would not recommend these. Buy the real Vince Camuto versions of these instead.</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
-      <c r="N3" s="5" t="n"/>
-      <c r="O3" s="5" t="n"/>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki "süper yumuşak konfor" ve "kolay yürüyüş/tüm gün mutlu ayaklar" vaatlerine karşılık; 2 farklı müşteri ayakkabının üretim hatalı (topuğa batan parça) olduğunu ve giyildiği an ayağı acıtıp çok rahatsız ettiğini (Kalite) belirterek konfor iddiasını çürütmüştür. Gıcırdama, sim dökülmesi, kayış kopması ve dengesizlik gibi diğer tüm şikayetler tekil kaldığı için elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="300" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -2883,19 +3892,39 @@
 3) [2★] Two Stars — Disappointed. Looking for someone wearing smaller size to gift thé pair.</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="300" customHeight="1">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Sayfada satılan standart koşu ayakkabısı beklentisine karşılık; 2 farklı müşteri ürünün kalıbının dar olduğunu ve beklenenden daha küçük numaraya uyduğunu (Beden/Kalıp) belirterek beden uyumsuzluğunu doğrulamıştır. İkinci el/kirli ürün gönderimi şikayeti tamamen satıcı hatası olduğu için elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="409.6" customHeight="1">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
@@ -2939,19 +3968,47 @@
 14) [1★] Not as well made as my others — Nothing like the pair Im replacing very disappointed</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="300" customHeight="1">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Sayfadaki "ortopedik yastıklama (EVA)", "benzersiz konfor" ve "kaymaz taban" vaatlerine karşılık; 6 yorum ürünün çok sert plastikten yapıldığını ve ayakları şiddetle ağrıttığını (Malzeme/Kalite), 3 yorum tabanın kaygan (slick/slippery) olduğunu (Kalite), 3 yorum ise geniş bedenlerin orantısız derecede devasa (iki ayak sığacak kadar) olduğunu (Beden/Kalıp) belirterek temel iddiaları çürütmüştür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="350" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
@@ -2984,19 +4041,39 @@
 4) [1★] Small for sizing — smaller than sizes say. Wife used the husband's socks.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="300" customHeight="1">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "sıkmayan uyum (non-constrictive)" ve "XXXL Bariatrik" beden vaatlerine karşılık; 3 yorum çorabın boğaz/bilek kısmının çok sıkı olduğunu (hatta kullanmak için kesilmesi gerektiğini) ve kalıpların bariatrik bir ürüne göre küçük olduğunu (Beden/Kalıp) belirterek temel iddiaları çürütmüştür. Yanlış ürün/beden gönderimi ve tekil dikiş şikayetleri elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="380" customHeight="1">
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
@@ -3038,17 +4115,45 @@
 12) [1★] They were small I would get three size bigger — To small got them for my lil one and they did not fit we’re three size to small</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "mükemmel uyum (fit) için ince ayar yapıyoruz" vaadine karşılık; 7 yorum kalıbın giyilemeyecek derecede orantısız olduğunu (belin 8 beden kadar dar, boyun 14-16 beden kadar uzun) belirterek (Beden/Kalıp), 2 yorum ise yıkanmasına rağmen geçmeyen ağır bir kimyasal koku olduğunu (Malzeme/Kalite) belirterek temel iddiaları çürütmüştür. Kullanılmış ürün ve tekil eksik düğme şikayetleri elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="300" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -3094,19 +4199,59 @@
 14) [2★] Not a cotton blend. — This dress looked very pretty when I received it, but I could tell from the feel of the material that this was not the cotton blend the description promised. I made the purchase for an outdoor summer event and I don't think it would wear well in the heat.</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="300" customHeight="1">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "A-kesim kum saati silüeti", "inanılmaz kumaş kalitesi" ve "pamuk" vaatlerine karşılık; 8 yorum malzemenin çok ince, kaşındırıcı ve ucuz hissettirdiğini (Malzeme/Kalite), 5 yorum elbisenin çuval gibi sarktığını ve görseldeki A-kesimle alakası olmadığını (Görsel/Beden/Kalıp), 2 yorum ilk yıkamada ürünün tüylenip söküldüğünü (Dayanıklılık), 2 yorum ise renklerin hatalı geldiğini (Renk) belirterek ana iddiaları tamamen çürütmüştür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="409.6" customHeight="1">
       <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
@@ -3150,17 +4295,49 @@
 15) [2★] Way to big and not body fitting like in the picture — I really really wanted to like this jacket, seeing pictures of other people wearing it, it looked good... not the one I got, the color is pretty but the jacket is just not right, it looks like I’m wearing a cute colored sack of potatoes 😂. I got a medium and it looks huuuge on me, I’m usually a medium with other brands. Also while opening it, one of the Velcroes came undone, so that was a bummer too. Maybe I just didn’t have luck with this one jacket since other people seemed to like it so much.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "etkileyici termal yalıtım" ve "tam fermuar koruması" vaatlerine karşılık; 5 yorum fermuarların hiç kapanmadığını veya hemen kırıldığını (Dayanıklılık/Kalite), 4 yorum kalıpların tabloda yazılandan inçlerce daha geniş, devasa ve çuval gibi olduğunu (Beden/Kalıp/Görsel), 2 yorum ise montun kayak yaparken veya hafif soğukta bile sıcak tutmadığını (Kalite) belirterek ana iddiaları tamamen çürütmüştür. Kullanılmış ve defolu ürün şikayetleri elenmiştir.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="300" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -3204,19 +4381,47 @@
 15) [2★] dont buy — i bought them 2 times 1st time ripet in a week 2nd time ripet 2weeks later</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="300" customHeight="1">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "%100 hakiki deri", "sağlam/dayanıklı" ve kauçuk taban vaatlerine karşılık; 3 yorum tabanın düşmeye sebep olacak kadar kaygan ve tehlikeli olduğunu (Kalite), 3 yorum ayakkabının birkaç hafta/ay içinde çatlayıp yırtıldığını (Dayanıklılık), 2 yorum ise yüzeyin ilk kullanımda sentetik gibi soyulup döküldüğünü (Malzeme) belirterek tüm temel iddiaları çürütmüştür. Tutarsız beden şikayetleri ve kullanılmış ürün gönderimi elenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="365" customHeight="1">
       <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
@@ -3253,24 +4458,53 @@
 9) [1★] Cheap Quality. Not worth the money. — Very poor stitching. The cloth material is not good. Not worth the money. Cant return it as I already wore it once in an emergency situation. Will appreciate if the seller returns half of the money.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="5" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>Sayfanın "göz alıcı tasarımcı işi elbise" vaadine karşılık; 3 yorum ürünün fotoğraftaki tasarımla hiç alakası olmadığını (Görsel), 3 yorum bedenlerin tutmadığını ve dar kalıplı olduğunu (Beden/Kalıp), 2 yorum ise kumaşın/dikişlerin çok ucuz ve kötü kalitede olduğunu (Malzeme/Kalite) belirterek ana estetik iddiaları tamamen çürütmüştür. Satıcının kullanılmış/lekeli ürün göndermesi ve iade politikası şikayetleri elenmiştir.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="E2:E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Evet,Hayır"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="E2:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Evet,Hayır"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:M11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Faz 4: 40 ürün gold etiketleme tamamlandı
- Etiketleme kuralları sürüm 2: tek konu kuralı, tip tanımları ve öncelik,
  'somut iddia' tanımı, kullanılmış ürün gönderimi = satıcı hatası
- 40 ürün yeni kurallarla yeniden gözden geçirildi (29 ürün, 91 alan değişti;
  data/gold/gozden_gecirme_degisiklikler.csv)
- Altın standart: 36 gap var / 4 yok, 62 tip etiketi (data/gold/gold_40.csv)
- kapsam.md 2.1: ana metrik gap tipi micro-F1, bootstrap güven aralığı,
  sınırlılıklar ve revizyon notları güncellendi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gold/etiketleme.xlsx
+++ b/data/gold/etiketleme.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,10 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -75,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -90,6 +94,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,18 +460,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ETİKETLEME TALİMATI</t>
-        </is>
-      </c>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>ETİKETLEME TALİMATI (kurallar sürüm 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -482,6 +490,9 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -524,92 +535,230 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   NOT: 'Çelişki yok' bir veri sorunu DEĞİLDİR. O durumda veri_uygun = Evet, gap_var = Hayır yazılır.</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1) gap_var: Evet / Hayır</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2) Konu sütunları: çelişki hangi konudaysa o sütuna X koy (birden fazla olabilir).</t>
+          <t>1) gap_var: Evet / Hayır</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Kural: Bir konu ancak EN AZ 2 yorum o sorundan bahsediyorsa işaretlenir.</t>
+          <t>2) Konu sütunları: çelişki hangi konudaysa o sütuna X koy (birden fazla olabilir).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3) seviye:</t>
+          <t xml:space="preserve">   Kural: Bir konu ancak EN AZ 2 yorum o sorundan bahsediyorsa işaretlenir.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Yüksek = Sayfa açıkça bir şey iddia etmiş, yorumlar tersini söylüyor (ör. 'su geçirmez' yazıyor, 'su aldı' diyorlar)</t>
+          <t xml:space="preserve">   TEK KONU KURALI: Bir şikayet yalnızca TEK konuya sayılır. Her konunun KENDİ en az 2 yorumu olmalı;</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Orta   = Sayfa o konuda bilgi vermemiş, yorumlar şikayet ediyor (ör. beden bilgisi yok, 'küçük geldi' diyorlar)</t>
+          <t xml:space="preserve">   aynı yorumlar iki konuyu birden desteklemek için kullanılamaz.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Yok    = Çelişki yok (gap_var = Hayır ise seviye de Yok)</t>
+          <t xml:space="preserve">   Konu tanımları:</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4) not: Neden bu kararı verdin, 1 cümle.</t>
+          <t xml:space="preserve">   - Beden/Kalıp:  ölçü, kalıp, oturuş</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Renk:         renk farklı veya soluk</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SAYILMAYANLAR: kargo/paketleme, satıcı/iade süreci, 'beğenmedim' gibi kişisel zevk, tek seferlik arıza (1 yorum).</t>
+          <t xml:space="preserve">   - Görsel:       fotoğraftaki görünümden farklı (renk hariç)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TEKRARLAR: Birebir aynı yorumlar script tarafından zaten ayıklandı. Yine de aynı kişinin neredeyse aynı yorumunu görürsen tek say.</t>
+          <t xml:space="preserve">   - Malzeme:      kumaşın/materyalin özelliği (ince, şeffaf, plastik gibi, su geçirmiyor, kaşındırıyor, sert)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Dayanıklılık: zamanla bozulma (X kullanım/yıkama sonra söküldü/yırtıldı)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ÖRNEK: Sayfa 'Waterproof leather boot' diyor; 2 yorum 'su aldı', 1 yorum 'kargo geç'.</t>
+          <t xml:space="preserve">   - Kalite:       SADECE ilk günden işçilik/üretim hatası (dikiş, düğme, fermuar, defolu/lekeli geliş)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">        -&gt; gap_var = Evet | Malzeme = X (su geçirmezlik malzeme iddiası) | seviye = Yüksek | not: 'Su geçirmez diyor, 2/2 ilgili yorum su aldı diyor'</t>
+          <t xml:space="preserve">                   ve somut sebep belirtmeyen genel 'cheap' / 'poor quality'</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Eksik Bilgi:  sayfada bilginin hiç olmaması</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Öncelik: Şikayet birden fazla konuya uyuyorsa en spesifik olana gider (Malzeme ve Dayanıklılık, Kalite'den önce).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3) seviye:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Yüksek = Sayfada ürüne özgü SOMUT bir iddia var ve yorumlar bu iddiayla DOĞRUDAN çelişiyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            (somut iddia: ölçü aralığı, kalıp uyarısı, materyal, 'waterproof', 'memory foam', renk adı vb.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Orta   = Sayfa o konuda bilgi vermemiş VEYA sadece genel pazarlama dili kullanmış, yorumlar şikayet ediyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            (genel pazarlama dili iddia sayılmaz: 'high quality', 'premium', 'perfect fit', markanın her üründe kullandığı metin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Renk:    renk adı var ve şikayet 'soluk/donuk' ise Orta; başka renk geldiyse Yüksek</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Yok    = Çelişki yok (gap_var = Hayır ise seviye de Yok)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Birden fazla konu varsa en yüksek seviye yazılır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>4) not: Neden bu kararı verdin, 1 cümle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SAYILMAYANLAR: kargo/paketleme, satıcı/iade süreci, 'beğenmedim' gibi kişisel zevk, tek seferlik arıza (1 yorum).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Kullanılmış/iade edilmiş ürün gönderimi satıcı hatasıdır, sayılmaz; hasarlı/delikli/lekeli/defolu YENİ ürün Kalite'dir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TEKRARLAR: Birebir aynı yorumlar script tarafından zaten ayıklandı. Yine de aynı kişinin neredeyse aynı yorumunu görürsen tek say.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ÖRNEK: Sayfa 'Waterproof leather boot' diyor; 2 yorum 'su aldı', 1 yorum 'kargo geç'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        -&gt; gap_var = Evet | Malzeme = X (su geçirmezlik malzeme iddiası) | seviye = Yüksek | not: 'Su geçirmez diyor, 2/2 ilgili yorum su aldı diyor'</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>ÖNEMLİ: Bu dosyayı bitirip GitHub'a commit etmeden yapay zeka sistemini ÇALIŞTIRMA.</t>
         </is>
@@ -843,19 +992,23 @@
         </is>
       </c>
       <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n"/>
       <c r="M3" s="4" t="n"/>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "rahat" kargo pantolon vaadine ve sunduğu beden ölçülerine karşılık, 5 farklı yorum ürünün belirtilen bedenlerden çok küçük olduğunu ve "skinny jean" gibi aşırı dar bir kalıbı olduğunu belirterek iddiayı çürütmüştür. Fermuar, yıkamada çekme, kaşındıran kumaş ve eksik parça (sadece pantolon gelmesi) şikayetleri "en az 2" kuralını sağlamadığı için elenmiştir.</t>
+          <t>Beden/Kalıp: 7 yorum (#2, #4, #5, #6, #7, #10, #11) küçük/dar kalıp bildiriyor. Verilen sayfa metninde somut beden ölçüsü bulunmadığından seviye Orta. Görsel: 3 yorum (#9, #12, #14) görselin tam takım beklentisi yarattığını, yalnız pantolon geldiğini bildiriyor; bu şikayetler eksik gönderim değil, görsel sunum uyuşmazlığı olarak değerlendirildi. Diğer şikayet grupları iki yorum eşiğini sağlamıyor.</t>
         </is>
       </c>
     </row>
@@ -903,29 +1056,29 @@
           <t>Evet</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M4" s="4" t="n"/>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "esnek, bedeni saran slim kalıp" ve "parti taytı" vaatlerine karşılık; 6 yorum pulların birbirine takıldığını, döküldüğünü ve bedeni çizdiğini (Kalite), 3 yorum ise kalıbın sarmadığını, belin gevşek ve ağın orantısız uzun olduğunu (Beden/Kalıp) belirterek iddiaları çürütmüştür. Tekil dikiş söküğü şikayeti elenmiştir.</t>
+          <t>Malzeme: 3 yorum (#2, #4, #8) pulların takılması, hareketi zorlaştırması veya cildi çizmesini bildiriyor. Dayanıklılık: 3 yorum (#5, #6, #7) kullanım sırasında dökülme, delinme veya yırtılma bildiriyor. Her yorum tek konuya sayıldı. Beden/Kalıp (#3) ve ilk teslimde dikiş kusuru (#1) tek yorumla sınırlı. “Stretchy” iddiasına açıkça karşı çıkan yalnız #4; tekrarlanan şikayetlerle doğrudan çelişen somut sayfa iddiası bulunmadığından seviye Orta.</t>
         </is>
       </c>
     </row>
@@ -983,12 +1136,12 @@
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>Sayfada turuncu renk belirtilmişken, 2 yorum rengin çok soluk ve donuk olduğunu belirterek beklenti çelişkisi oluşturmuştur (Renk); çorabın küçük olduğuna dair tekil şikayet elenmiştir.</t>
+          <t>Renk: 2 yorum (#1, #2) turuncunun donuk/soluk olduğunu bildiriyor. Sayfada “Orange” yazıyor; farklı renk geldiği belirtilmediğinden seviye Orta. Beden/Kalıp: küçük olma şikayeti (#3) tek yorumla sınırlı olduğundan işaretlenmedi.</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1215,12 @@
       <c r="M6" s="4" t="n"/>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın büyük bedenler için "kısıtlama yapmayan esneklik ve tüm gün rahatlık" vaadine karşılık; 4 yorum ağ boyunun kısa ve kalıbın çok dar olduğunu (Beden/Kalıp), 2 yorum ise ürünün giyildiği ilk saatlerde/günde yırtıldığını (Dayanıklılık) belirterek iddiaları çürütmüştür. Yanlış renk gönderimi ve tekil dikiş detayı şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 11 yorum (#1, #2, #4, #7, #8, #9, #10, #11, #12, #13, #15) dar/kısa gelme, kötü oturuş, kayma veya kalıp tutarsızlığı bildiriyor; verilen sayfada somut ölçü aralığı yok → Orta. Dayanıklılık: 2 yorum (#3, #5) ilk saat/gün kullanımında delinme/yırtılma bildiriyor; somut dayanıklılık vaadi yok → Orta. Her yorum tek konuya sayıldı. Fotoğraftan farklı dikiş yapısı (#6) tek yorumla sınırlı; #14 kişisel itiraz olduğundan elendi.</t>
         </is>
       </c>
     </row>
@@ -1117,29 +1270,25 @@
           <t>Evet</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M7" s="4" t="n"/>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Sayfanın "uzun süreli kullanıma uygun, ferah ve klasik Crocs rahatlığı" vaatlerine karşılık; 2 yorum ürünün iç astarı olmaması ve sert yapısı nedeniyle bilek kemiklerine sürttüğünü, kanayan yaralara ve su toplamalarına yol açtığını (Beden/Kalıp, Kalite) belirterek iddiaları çürütmüştür. 1 aydan kısa sürede yıpranma, kupon eksikliği ve genel kalite düşüşü şikayetleri tekil kaldığı için elenmiştir.</t>
+          <t>Dayanıklılık: 2 yorum (#1, #2) kullanım sırasında erken yırtılma/bozulma bildiriyor; #1’deki birden fazla çift deneyimi tek yorum sayıldı. Sayfada somut kullanım ömrü veya yırtılmaya dayanıklılık iddiası yok → Orta. Astarsız kauçuk iç yüzeyin sürtmesi (#3) Malzeme, bileğe baskı yapan kalıp (#4) Beden/Kalıp olarak ayrı değerlendirildi; her biri tek yorum olduğundan işaretlenmedi. Kupon şikayeti (#5) elendi.</t>
         </is>
       </c>
     </row>
@@ -1192,11 +1341,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="L8" s="4" t="n"/>
       <c r="M8" s="4" t="n"/>
       <c r="N8" s="4" t="inlineStr">
         <is>
@@ -1205,7 +1350,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın başlığındaki "Fleece" (polar) vaadine karşılık; 2 yorum ürünün polar olmadığını ve çok ince bir pamuklu olduğunu (Malzeme), 3 yorum ise ürünün giyildiği anda/ilk günde dikişlerinden yırtıldığını ve deliklerle geldiğini (Dayanıklılık/Kalite) belirterek iddiaları çürütmüştür. Tekil dar kalıp şikayeti elenmiştir.</t>
+          <t>Malzeme: 2 yorum (#2, #4) kumaşın polar olmadığını, ince ve astarsız olduğunu bildiriyor; başlıktaki “Fleece” iddiasıyla doğrudan çelişiyor → Yüksek. Kalite: 2 yorum (#3, #5) dikiş boyunca delikler veya teslim alındığı gün görülen yırtık bildiriyor. Kullanımda yırtılma (#1) tek yorum olduğundan Dayanıklılık işaretlenmedi. #2 yalnız Malzeme altında sayıldı.</t>
         </is>
       </c>
     </row>
@@ -1378,32 +1523,24 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Evet</t>
+          <t>Hayır</t>
         </is>
       </c>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="n"/>
       <c r="M11" s="4" t="n"/>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>Orta</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "yüksek kalite" vaadine ve sunduğu görsellere karşılık, 2 farklı müşteri gelen ürünün fotoğraftakine benzemediğini ve kalitesiz/tuhaf bir kumaşı olduğunu belirterek iddiaları çürütmüştür (Görsel, Kalite). Dar kalıp, kimyasal koku ve renk şikayetleri "en az 2" kuralını sağlamadığı için elenmiştir.</t>
+          <t>Kimyasal koku ile “tuhaf kumaş” aynı sorun değil. Diğer yorumlarda da iki bağımsız yorumla doğrulanan, yeterince açık ortak şikayet yok.</t>
         </is>
       </c>
     </row>
@@ -1472,21 +1609,13 @@
         </is>
       </c>
       <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="L12" s="4" t="n"/>
       <c r="M12" s="4" t="n"/>
       <c r="N12" s="4" t="inlineStr">
         <is>
@@ -1495,7 +1624,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "Relaxed fit, dayanıklı ve kanvas" vaatlerine karşılık; 7 yorum ürünün çok küçük/kısa olduğunu (Beden/Kalıp), 4 yorum anında yırtıldığını/dikişlerin kalitesizliğini (Dayanıklılık/Kalite), 2 yorum kağıt gibi olup kanvas olmadığını (Malzeme) ve 2 yorum rengin farklı/koyu geldiğini (Renk) belirterek temel iddiaları çürütmüştür</t>
+          <t>Beden/Kalıp: 9 yorum (#2, #3, #6, #9, #10, #11, #12, #14, #15); özellikle #2, #3, #9 ve #14’teki dar/küçük kalıp şikayetleri sayfanın “Relaxed fit” iddiasıyla çelişiyor → Yüksek. Renk: 2 yorum (#8, #13) koyuluk/renk farkı bildiriyor. Malzeme: 2 yorum (#4, #7) kâğıt gibi kumaş veya kanvas olmama şikayeti bildiriyor. Genel kalite şikayeti (#1) ve ilk giyimde yırtılma (#5) ayrı konularda tek yorumla sınırlı. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -1612,12 +1741,12 @@
       <c r="M14" s="4" t="n"/>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın rahatlık ve beden/genişlik uyumu vaatlerine karşılık, 3 farklı yorum ayakkabının beklenen numaralardan çok daha küçük olduğunu belirterek iddiayı çürütmüştür (Beden/Kalıp). Yastıklama eksikliği şikayeti tekil kaldığı, yanlış eşleştirilmiş genişlik şikayeti ise satıcı hatası olduğu için elenmiştir.</t>
+          <t>Beden/Kalıp: 3 yorum (#1, #2, #3) küçük/dar gelme bildiriyor. Sayfadaki “perfect fit” ve beden/genişlik seçenekleri ifadeleri genel marka pazarlaması; ürüne özgü somut ölçü/kalıp iddiası bulunmadığından seviye Orta. Yastıklama eksikliği (#2) tek yorumla sınırlı ve ayrıca sayılmadı. Sol ve sağ ayakkabının farklı genişlikte gelmesi (#4) tekil çift eşleştirme kusuru olarak ayrıldı.</t>
         </is>
       </c>
     </row>
@@ -1667,11 +1796,7 @@
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J15" s="4" t="n"/>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="4" t="inlineStr">
         <is>
@@ -1681,12 +1806,12 @@
       <c r="M15" s="4" t="n"/>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "%100 Deri" ve hareketli yaşama uygunluk vaatlerine karşılık; 4 farklı yorum derinin çok kısa sürede (1.5 - 2 ay) çatladığını ve yırtıldığını (Dayanıklılık), 3 yorum ise ayakkabının çok sert, ağır ve rahatsız olduğunu (Kalite) belirterek temel iddiaları çürütmüştür. Tekil kalıp (büyük) şikayeti elenmiştir.</t>
+          <t>Dayanıklılık: 4 yorum (#3, #4, #5, #7) çatlama, yırtılma/soyulma veya kısa kullanım ömrü bildiriyor. “%100 deri” içerik iddiası, çatlama şikayetleriyle doğrudan çürütülmüyor; somut kullanım ömrü vaadi bulunmadığından seviye Orta. Malzeme sertliği/ağırlığı (#2) ve kalıp/oturuş sorunu (#1) ayrı konularda tek yorumla sınırlı. #1 ve #6’daki gelecekte bozulma tahminleri Dayanıklılık sayısına eklenmedi.</t>
         </is>
       </c>
     </row>
@@ -1807,11 +1932,7 @@
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
@@ -1821,12 +1942,12 @@
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın güvenlik amaçlı "vücudu saran kalıp (snug fit)" vaadine karşılık, 4 yorum ürünün kollarının/bacaklarının orantısız derecede kısa ve giyilemeyecek kadar küçük olduğunu (Beden/Kalıp); 2 yorum ise dikişlerin ilk birkaç kullanımda anında söküldüğünü (Dayanıklılık/Kalite) belirterek beklentileri tamamen çürütmüştür. Leke ve yıkama sonrası sarkma şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 4 yorum (#1, #4, #5, #8) küçük gelme, kısa kol veya yetersiz örtücülük bildiriyor. “Snug fit” dar oturuş uyarısı; şikayetlerle doğrudan çelişen somut ölçü iddiası yok → Orta. Dayanıklılık: 3 yorum (#3, #6, #7) yıkama sonrası solma/şekil kaybı veya kullanımda dikiş sökülmesi bildiriyor. Yıkama sonrası bozulma yalnız #3’te açık; #4’teki çekme tahmini sayılmadı. Lekeli/eksik baskılı geliş (#2) tek yorum olduğundan Kalite işaretlenmedi. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -1895,11 +2016,7 @@
       </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J18" s="4" t="n"/>
       <c r="K18" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -1918,7 +2035,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "iç göstermez, derin squata uygun, dayanıklı ve destekleyici" vaatlerine karşılık; 8 yorum ürünün ilk kullanımlarda dikişlerinden yırtıldığını (Dayanıklılık), 3 yorum eğilirken tamamen iç gösterdiğini (Malzeme), 4 yorum kalıbın çok küçük olduğunu (Beden/Kalıp) ve 2 yorum sütyenin desteklemediğini (Kalite) belirterek tüm ana iddiaları çürütmüştür. Açık paket ve koku şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 5 yorum (#2, #3, #5, #12, #14) beden uyumsuzluğu bildiriyor. Malzeme: 2 yorum (#6, #7) ışıkta/eğilmede iç gösterdiğini belirtiyor; sayfanın “really non-see through” iddiasıyla doğrudan çelişiyor → Yüksek. Dayanıklılık: 7 yorum (#4, #8, #9, #10, #11, #13, #15) kullanımda veya yıkama sonrası yırtılma/dikiş açılması bildiriyor. #1’de kusurun oluşma zamanı belirsiz olduğundan Kalite/Dayanıklılık sayımına eklenmedi. Her yorum tek konuya sayıldı; tekrarlanan alışveriş deneyimleri ayrı yorum sayılmadı.</t>
         </is>
       </c>
     </row>
@@ -1967,11 +2084,7 @@
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J19" s="4" t="n"/>
       <c r="K19" s="4" t="n"/>
       <c r="L19" s="4" t="inlineStr">
         <is>
@@ -1986,7 +2099,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "dayanıklı (durable)" yapı ve "gün boyu güvenli tutuş (secure fit)" sağlayan cırt cırt vaatlerine karşılık; 2 yorum ürünün ilk kullanımlarda koptuğunu/parçalandığını (Dayanıklılık), diğer 2 yorum ise cırt cırtların çok kısa sürede yapışkanlığını yitirdiğini (Kalite) belirterek temel iddiaları çürütmüştür. Tekil dar/uzun kalıp şikayeti elenmiştir.</t>
+          <t>Dayanıklılık: 4 yorum (#1, #3, #4, #5). #1 ve #5 cırtların kullanım sonrası tutmadığını; #3 ve #4 ilk gün/birkaç kullanımda kırılma veya kayış kopması bildiriyor. Cırtların tutmaması, sayfanın cırtlı kapama için verdiği “more secure fit throughout the day” vaadiyle doğrudan çelişiyor → Yüksek. Sonradan oluşan işlev kaybı Kalite yerine Dayanıklılık altında toplandı. Uzun/dar kalıp şikayeti (#2) tek yorumla sınırlı.</t>
         </is>
       </c>
     </row>
@@ -2038,22 +2151,18 @@
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="n"/>
       <c r="L20" s="4" t="n"/>
       <c r="M20" s="4" t="n"/>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "aktif koşu pantolonu" ve "3 cep" vaatlerine karşılık; 3 yorum kalıbın aşırı küçük/orantısız olduğunu ve belden düştüğü için koşmayı engellediğini (Beden/Kalıp), 2 yorum ise ceplerin kullanılamayacak kadar küçük veya sahte olduğunu (Kalite) belirterek ana iddiaları çürütmüştür. Tekil malzeme (kağıt gibi dış kumaş) şikayeti elenmiştir.</t>
+          <t>Beden/Kalıp: 2 yorum (#1, #2) bel-bacak orantısızlığı, kayma veya küçük beden bildiriyor. Sayfada “slim fit” uyarısı var; somut beden ölçüsü bulunmadığından seviye Orta. Her yorum tek konuya sayıldı. Küçük cep (#1), işlevsiz arka cep ve sert dış kumaş (#2) ayrıca konu desteğine eklenmedi. #3 ürünün torununa tam olduğunu söylüyor; somut şikayet içermediğinden sayılmadı.</t>
         </is>
       </c>
     </row>
@@ -2099,11 +2208,7 @@
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="n"/>
       <c r="L21" s="4" t="inlineStr">
         <is>
@@ -2113,12 +2218,12 @@
       <c r="M21" s="4" t="n"/>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın kauçuk tabanlı su ayakkabısı vaadine karşılık, 3 farklı yorum tabanın sadece 1-2 gün içinde delindiğini, aşındığını veya daha kullanılmadan iplerinin sökülerek parçalandığını (Dayanıklılık/Kalite) belirterek ürünün asgari işlevini çürütmüştür.</t>
+          <t>Dayanıklılık: 2 yorum (#1, #3) iki kullanımda delinme veya bir günde taban aşınması bildiriyor. Sayfada somut aşınma/delinme direnci vaadi yok; “rubber sole” malzeme tanımı ve “waterproof” iddiası bu yorumlarla doğrudan çürütülmüyor → Orta. Kullanım öncesi taban ayrılması ve sökülmüş iplikler (#2) Kalite kapsamında tek yorum olduğundan işaretlenmedi.</t>
         </is>
       </c>
     </row>
@@ -2184,31 +2289,27 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="n"/>
       <c r="M22" s="4" t="n"/>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>Sayfadaki "Loose Fit" ibaresine rağmen 3 yorum ürünün 1-2 beden daha büyük/orantısız olduğunu (Beden/Kalıp); 3 yorum rengin görseldekiyle ilgisi olmayıp neredeyse siyah renkte geldiğini (Renk/Görsel); 4 yorum ise dikişlerin çok özensiz olduğunu ve hemen sökülüp delindiğini (Kalite/Dayanıklılık) belirterek beklentileri çürütmüştür. Satıcı/yanlış ürün, koku ve haksız malzeme şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 3 yorum (#1, #9, #11) büyük gelme bildiriyor; “loose fit” bol kesim tanımıyla doğrudan çelişki yok. Renk: 2 yorum (#5, #7) koyuluk/solukluk bildiriyor. Kalite: 3 yorum (#6, #8, #15) özensiz dikiş veya yırtık/delikli teslim bildiriyor. Malzeme: 3 yorum (#3, #4, #14) kaşındıran kumaş, kimyasal koku veya incelik bildiriyor. Kullanım sonrası bozulma (#2) tek yorum olduğundan Dayanıklılık işaretlenmedi. #10’un %100 pamuk iddiası verilen sayfayla uyuşmuyor; #12 ve #13 yanlış ürün/beden gönderimi kapsamında ayrıldı. Her yorum tek konuya sayıldı; somut sayfa iddiasıyla desteklenen doğrudan çelişki bulunmadığından seviye Orta.</t>
         </is>
       </c>
     </row>
@@ -2260,30 +2361,22 @@
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="L23" s="4" t="n"/>
       <c r="M23" s="4" t="n"/>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "dayanıklı yapı (durable construction)" vaadine karşılık; 2 yorum ürünün paketinden delik çıktığını veya yarım saatlik kullanımda delindiğini (Dayanıklılık/Kalite), 2 yorum da malzemenin çok ucuz ve ince olduğunu (Malzeme) belirterek ana iddiaları çürütmüştür. Tekil renk/desen ve dar baldır şikayetleri elenmiştir.</t>
+          <t>Malzeme: 2 yorum (#2, #3) iç gösterecek kadar ince kumaş bildiriyor. Sayfada kalınlık veya opaklık vaadi yok; kumaş “lightweight” olarak tanımlanıyor → Orta. Delikli teslim (#1) Kalite, yarım saat kullanımda delinme (#5) Dayanıklılık olarak ayrıldı; her biri tek yorum olduğundan işaretlenmedi. Baldır darlığı (#4) tek yorumla sınırlı. #2 yalnız Malzeme altında sayıldı.</t>
         </is>
       </c>
     </row>
@@ -2346,26 +2439,18 @@
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "premium pamuk" ve göğüs/omuzda "hafifçe dar (slightly slimmer) Custom Fit" vaatlerine karşılık; 4 yorum kalıbın aşırı küçük/orantısız olduğunu ve 3XL bedenin ancak bir çocuğa uyduğunu (Beden/Kalıp), 3 yorum ise kumaşın çok ucuz, ince ve kalitesiz hissettirdiğini (Kalite/Malzeme) belirterek ana iddiaları çürütmüştür. Satıcı hataları ve tekil renk şikayeti elenmiştir.</t>
+          <t>Beden/Kalıp: 3 yorum (#1, #3, #9) dar/küçük kalıp bildiriyor. Sayfada daha dar göğüs-omuz ve kısa boy uyarısı var; somut ölçüyle doğrudan çelişki doğrulanmadığından seviye Orta. İnce kumaş (#4) ve fazla kalın kumaş (#5) aynı sorunu desteklemediğinden Malzeme işaretlenmedi. Kullanılmış ürün gönderimi (#7) satıcı süreci olarak elendi. Hasarlı teslim (#6) ile genel düşük kalite (#10) aynı sorunu doğrulamadığından Kalite işaretlenmedi.</t>
         </is>
       </c>
     </row>
@@ -2428,11 +2513,7 @@
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
       <c r="L25" s="4" t="inlineStr">
         <is>
@@ -2442,12 +2523,12 @@
       <c r="M25" s="4" t="n"/>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "dolgulu lüks iç taban" ve "olağanüstü konfor" vaatlerine karşılık; 3 yorum tabanın krep gibi dümdüz olduğunu ve hiçbir destek sunmadığını (Kalite), 5 yorum kalıbın aşırı küçük/orantısız olduğunu (Beden/Kalıp), 2 yorum kısa sürede esneyip şeklinin bozulduğunu (Dayanıklılık) belirterek ana iddiaları çürütmüştür. Eşitsiz ayakkabı (defolu ürün) ve iade sorunları elenmiştir</t>
+          <t>Beden/Kalıp: 10 yorum (#1, #2, #3, #4, #7, #8, #9, #11, #12, #14) ölçü, oturuş veya ayak kavsi desteği sorunu bildiriyor. Dayanıklılık: 2 yorum (#10, #15) esneme/şekil kaybı bildiriyor. “Padded insole” kavis desteği vaadi değildir; dolgunun bulunmadığı açıkça belirtilmediğinden seviye Orta. Farklı büyüklükte tekler (#5) tekil Kalite şikayeti. #6 olumlu, #13 paketleme kaynaklı şikayet olarak ayrıldı. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -2645,11 +2726,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J28" s="4" t="n"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -2659,12 +2736,12 @@
       <c r="M28" s="4" t="n"/>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "zarif, midi-boy yün kaban" vaadine karşılık; 4 yorum ürünün bir çocuk kabanı kadar küçük ve orantısız olduğunu (Beden/Kalıp), 4 yorum yanlış renk geldiğini (Renk), 6 yorum kumaşın çok ucuz, ince, sert ve kalitesiz olduğunu (Malzeme/Kalite), 2 yorum ise kesiminin ve duruşunun fotoğrafla hiç alakası olmadığını (Görsel) belirterek tüm temel iddiaları çürütmüştür. Kargo ve iade şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 4 yorum (#5, #6, #11, #12) aşırı küçük kalıp bildiriyor. Renk: 4 yorum (#2, #7, #14, #15) beklenen maviden koyu/farklı ton bildiriyor; verilen sayfada yalnız “blue” yazıyor. Görsel: 2 yorum (#9, #13) kesim/döküm veya görünümün fotoğrafla uyuşmadığını belirtiyor. Malzeme: 2 yorum (#1, #10) sertlik/kaşıntı veya incelik bildiriyor. Genel kalite ifadesi (#3) tek yorum; #4 gerekçesiz, #8 teslimat şikayeti. Her yorum tek konuya sayıldı. Verilen somut sayfa iddialarıyla doğrudan çelişki doğrulanmadığından seviye Orta.</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2924,11 @@
           <t>Evet</t>
         </is>
       </c>
-      <c r="G31" s="4" t="n"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="inlineStr">
@@ -2855,7 +2936,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="K31" s="4" t="n"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -2869,7 +2954,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "hafızalı sünger konforu" ve "yüksek kalite" vaatlerine karşılık; 2 yorum süngerin anında çökerek terliğin ayaktan çıkmasına/kramp yapmasına sebep olduğunu (Kalite), 3 yorum ise iç tabanların birkaç ay içinde yırtılıp ürünün parçalandığını (Dayanıklılık) belirterek ana iddiaları çürütmüştür. Satıcı, kullanılmış ürün ve tekil defo şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 2 yorum (#5, #6) numara ölçülerinin aynı olması veya dar kalıp bildiriyor. Malzeme: 2 yorum (#1, #3) köpük tabanın hemen ezilip yastıklamayı yitirdiğini bildiriyor; uzun süreli konfor sağlayan “memory foam cushioned insoles” vaadiyle çelişiyor → Yüksek. Kalite: 3 yorum (#2, #7, #9) eşitsiz tekler, lekeli/kullanılmış teslim veya üretim kusuru bildiriyor. Dayanıklılık: 2 yorum (#10, #11) birkaç ayda yırtılma/parçalanma bildiriyor. #4’ün nedeni belirsiz; #8’deki ömür tahmini sayılmadı. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -2929,11 +3014,7 @@
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J32" s="4" t="n"/>
       <c r="K32" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -2948,7 +3029,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "ilave sıcaklık sağlayan termal takım" vaadine karşılık; 4 yorum malzemenin çok ince olduğunu ve çocukların suda titreyip morardığını (Malzeme/Kalite), 4 yorum ise ürünün gövdeden çok kısa ve belden bol olacak şekilde orantısız bir kesime sahip olduğunu (Beden/Kalıp) belirterek temel iddiaları çürütmüştür. Tekil yırtılma şikayeti elenmiştir.</t>
+          <t>Beden/Kalıp: 3 yorum (#1, #2, #6) büyük beden seçimine rağmen kısa/dar gövde veya bel-gövde orantısızlığı bildiriyor. Malzeme: 3 yorum; #3 kumaşın inceliğinden, #4 ve #7 yetersiz ısı yalıtımından şikayetçi. #4 ve #7 sayfanın termal koruma/ek sıcaklık vaadiyle çelişiyor → Yüksek. #3 suda denemediğinden termal performans çelişkisine kanıt sayılmadı. Nedeni belirsiz rahatsızlık (#5) ayrıldı; kullanımda delinme (#8) tek yorum olduğundan Dayanıklılık işaretlenmedi. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -2995,21 +3076,9 @@
         </is>
       </c>
       <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -3024,7 +3093,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>Sayfadaki görsel estetik beklentisine karşılık; 2 yorum rengin görseldeki gibi canlı olmadığını (Renk/Görsel), 3 yorum ise malzemenin çok ince, dayanıksız (flimsy) ve ucuz görünümlü olduğunu (Kalite/Malzeme) belirterek iddiaları çürütmüştür. Tekil gizli cep şikayeti elenmiştir.</t>
+          <t>Malzeme: 2 yorum (#2, #3) ince kumaş veya ceplerde gevşek/flimsy kumaş nedeniyle dağınık görünüm bildiriyor. Sayfa kumaşı “lightweight” olarak tanımlıyor; somut kalınlık/tokluk vaadi bulunmadığından seviye Orta. #1 renk şikayetine ayrıldı ve tek yorumla sınırlı kaldı. #2’nin renk, #3’ün görsel şikayeti ikinci kez sayılmadı. Somut işçilik kusuru veya kullanımda bozulma desteği bulunmuyor.</t>
         </is>
       </c>
     </row>
@@ -3147,31 +3216,19 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
       <c r="L35" s="4" t="n"/>
       <c r="M35" s="4" t="n"/>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "nefes alabilir, yumuşak kumaş" vaadine karşılık; 7 yorum kumaşın plastik gibi hissettirdiğini, nefes almadığını ve çok kalitesiz/ince olduğunu (Malzeme/Kalite), 4 yorum kalıpların standart dışı ve aşırı tutarsız (L'nin 3X, XXL'nin M gibi) olduğunu (Beden/Kalıp), 2 yorum ise rengin soluk/tozlu görünüp görselle uyuşmadığını (Renk/Görsel) belirterek ana iddiaları çürütmüştür. Kullanılmış ürün/satıcı şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 5 yorum (#5, #9, #11, #14, #15) küçük/kısa gelme bildiriyor; #4 ve #13 ayrıca büyüklük/kalıp tutarsızlığı içeriyor. Sayfada özel beden tablosunu kullanma uyarısı var, ancak verilen metinde somut ölçü yok → Orta. Renk: 2 yorum (#1, #12) siyahın soluk/tozlu veya koyu gri görünmesini bildiriyor → Orta. Kullanılmış ürün gönderimleri (#3, #8) satıcı süreci olarak elendi; Kalite işaretlenmedi. #2, #7 ve #10 farklı malzeme sorunları bildirdiğinden Malzeme işaretlenmedi. Görsel fark (#6) tek yorumla sınırlı.</t>
         </is>
       </c>
     </row>
@@ -3240,12 +3297,12 @@
       <c r="M36" s="4" t="n"/>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>Sayfadaki "2 beden küçük kalıptır" uyarısına rağmen; incelenen 10 yorumun 10'u da kalıbın aşırı derecede küçük ve tutarsız olduğunu, 2 veya daha fazla beden büyük almanın bile ayakkabıyı giymek için yetersiz kaldığını (Beden/Kalıp) belirterek sayfanın temel beden yönlendirmesini çürütmüştür.</t>
+          <t>Beden/Kalıp: 15 yorum (#1–#15) küçük kalıp veya numara büyütme ihtiyacı bildiriyor. Sayfa normal ayakkabıya göre 2 numara küçük kalıp uyarısı içeriyor. İki numara büyük almasına rağmen yetersiz kaldığını açıkça bildiren #5; #9 ve #15 uyarıyla uyumlu, #4 ve #12 yalnız bir numara büyütmüş. #11’deki 2–2,5 numara ifadesi ve #3/#7’deki numara geçişleri ikinci bir kesin çelişki olarak sayılmadı. Seviye Orta.</t>
         </is>
       </c>
     </row>
@@ -3305,11 +3362,7 @@
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J37" s="4" t="n"/>
       <c r="K37" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -3328,7 +3381,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "nefes alabilen file", "dayanıklı kumaş" ve "rahat uyum" vaatlerine karşılık; 8 yorum ürünün nem emmediğini, plastik poşet gibi terletip koku yaptığını (Malzeme/Kalite), 3 yorum bacakları aşırı sıktığını ve kalıpların tutarsız olduğunu (Beden/Kalıp), 3 yorum ise birkaç kullanımda delinip parçalandığını (Dayanıklılık) belirterek temel spor iddialarını çürütmüştür. Kargo ve okuma hatası şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 3 yorum (#5, #10, #11) sıkılık/kalıp tutarsızlığı bildiriyor. Malzeme: 8 yorum (#2, #4, #6, #7, #9, #13, #14, #15) terleme, nem veya koku şikayeti içeriyor; özellikle #2, #6, #7, #9, #13 ve #15 sayfanın “breathable mesh” iddiasıyla çelişiyor → Yüksek. Dayanıklılık: 2 yorum (#8, #12) birkaç kullanımda parçalanma/delinme bildiriyor. Hasarlı teslim (#1) tek yorum olduğundan Kalite işaretlenmedi. #3’ün kısa çorap beklentisi verilen sayfayla uyuşmuyor. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -3390,11 +3443,7 @@
       </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J38" s="4" t="n"/>
       <c r="K38" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -3408,12 +3457,12 @@
       <c r="M38" s="4" t="n"/>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın konforlu adım ve dayanıklı kayış/taban vaatlerine karşılık; 8 yorum ürünün aşırı dar ve küçük olduğunu (Beden/Kalıp), 3 yorum kayış malzemesinin aşındırıcı olup ayağı soyduğunu (Malzeme/Kalite), 3 yorum ise tabanların haftalar/aylar içinde tamamen koptuğunu (Dayanıklılık) belirterek temel ürün işlevlerini çürütmüştür. İade ve koku şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 8 yorum (#1, #2, #5, #6, #10, #11, #12, #15) dar/küçük kalıp veya yüksek kavis baskısı bildiriyor. Malzeme: 3 yorum (#3, #7, #13) aşındırıcı temas yüzeyi, koku veya cilt rahatsızlığı bildiriyor. Dayanıklılık: 3 yorum (#4, #8, #9) taban ayrılması, kayış liflenmesi veya topuk aşınması bildiriyor. Dolgulu taban ve kalın deri/kumaş kayış tanımları bu şikayetlerle doğrudan çürütülmüyor; somut ölçü, pürüzsüzlük veya kullanım ömrü vaadi yok → Orta. #14 iade şikayeti olarak elendi. Her yorum tek konuya sayıldı.</t>
         </is>
       </c>
     </row>
@@ -3466,23 +3515,19 @@
         </is>
       </c>
       <c r="H39" s="4" t="n"/>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I39" s="4" t="n"/>
       <c r="J39" s="4" t="n"/>
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="n"/>
       <c r="M39" s="4" t="n"/>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "vücut hatlarınızı gösteren A-kesim" ve "zarif duruş" vaatlerine karşılık; 2 yorum elbisenin tamamen şekilsiz, kutu gibi ve aşırı bol olduğunu (Beden/Kalıp), 2 yorum ise boyunun modeldekinden uzun ve tuhaf durduğunu (Görsel) belirterek temel estetik iddiaları çürütmüştür. Tekil yaka ve kol tasarımı şikayetleri elenmiştir.</t>
+          <t>Beden/Kalıp: 2 yorum (#1, #2) kutu gibi, şekilsiz veya aşırı bol oturuş bildiriyor. Sayfa “loose fit”, “loose A-line” ve “roomy” ifadeleriyle bol kesimi açıklıyor; somut ölçü iddiasıyla doğrudan çelişki yok → Orta. #2’deki modelden uzun görünme ayrıca Görsel için sayılmadı. #3’ün boy, yaka, kabarık kol ve desen eleştirileri kişisel beğeni niteliğinde; sayfadan farklı ürün geldiğine dair açık karşılaştırma içermiyor.</t>
         </is>
       </c>
     </row>
@@ -3541,12 +3586,12 @@
       <c r="M40" s="4" t="n"/>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>Yüksek</t>
+          <t>Orta</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>Sayfanın "optimal destek sağlayan bel bandı" vaadine ve sunduğu beden ölçülerine karşılık; 3 yorum beden tablosunun tamamen yanıltıcı olduğunu, şortun aşırı küçük üretildiğini ve esnemeyen bel bandı yüzünden ürünün (örneğin 36 inç bele XL bedenin) kalçadan dahi geçmediğini (Beden/Kalıp) belirterek temel iddiaları çürütmüştür.</t>
+          <t>Beden/Kalıp: 3 yorum (#1, #2, #3) aşırı dar kalıp veya yanıltıcı beden tablosu bildiriyor. Verilen sayfa metninde somut beden ölçüsü/tablosu yok; #2’deki “XL 36–38 inç” bilgisi yorumcunun başka siteye atfı olduğundan sayfa iddiası olarak doğrulanamadı. “Optimal support” belirli beden uyumu veya esneklik garantisi değil. Mevcut kanıtla seviye Orta.</t>
         </is>
       </c>
     </row>

</xml_diff>